<commit_message>
:up: algumas questoes respondidas - port
</commit_message>
<xml_diff>
--- a/banco_de_dados/caderno_anotacoes.xlsx
+++ b/banco_de_dados/caderno_anotacoes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1383,6 +1383,34 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>58</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>22/09/2026 10:24</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>5927</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Morfologia</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>fazer um resumo sobre as regras de colocação dos pronomes átonos (principalmente evidenciando a ordem de prioridade)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>